<commit_message>
update summer chinook brood table to add 24 and add covariates table
</commit_message>
<xml_diff>
--- a/data-raw/data/SummerChinook.xlsx
+++ b/data-raw/data/SummerChinook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa.sharepoint.com/sites/DFW-TeamFPColumbiaRiverManagementUnit953/Shared Documents/Data and Analysis Tools/Forecasting/Cox_forecast_ensemble/Data/2024/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa.sharepoint.com/sites/DFW-TeamWashingtonOregonColumbiaRiverFisheriesJointManage546/Shared Documents/General/USvsOR/Forecasting/2025/TAC_SprSum25/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{E77DB1D3-E046-4B57-A9F7-B64073277D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{049A63D0-6588-4851-B8EE-6B0011E17C02}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{E77DB1D3-E046-4B57-A9F7-B64073277D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B0BAD83-2032-4DF3-9159-35F86A8B9390}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{820E0690-656E-44D1-9707-41A341FF10ED}"/>
+    <workbookView xWindow="8208" yWindow="684" windowWidth="17280" windowHeight="8964" xr2:uid="{820E0690-656E-44D1-9707-41A341FF10ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="7">
   <si>
     <t>BroodYear</t>
   </si>
@@ -63,7 +63,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -82,8 +82,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -93,12 +99,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF595959"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -165,9 +165,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -186,9 +187,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -226,7 +227,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -332,7 +333,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -474,7 +475,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -482,10 +483,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11D27B93-ADEE-4F6A-B5E0-B0D968FFF1EF}">
-  <dimension ref="A1:F38"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:K39"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -505,13 +506,13 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1984</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="10"/>
+      <c r="D2" s="8"/>
       <c r="E2" s="6">
         <v>1549</v>
       </c>
@@ -519,12 +520,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1985</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="C3" s="10"/>
+      <c r="C3" s="8"/>
       <c r="D3" s="7">
         <v>9378</v>
       </c>
@@ -535,7 +536,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1986</v>
       </c>
@@ -555,7 +556,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>1987</v>
       </c>
@@ -575,7 +576,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>1988</v>
       </c>
@@ -595,7 +596,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1989</v>
       </c>
@@ -615,7 +616,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1990</v>
       </c>
@@ -635,7 +636,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>1991</v>
       </c>
@@ -655,7 +656,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1992</v>
       </c>
@@ -675,7 +676,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>1993</v>
       </c>
@@ -695,7 +696,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>1994</v>
       </c>
@@ -715,7 +716,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>1995</v>
       </c>
@@ -735,7 +736,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1996</v>
       </c>
@@ -755,7 +756,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>1997</v>
       </c>
@@ -775,7 +776,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>1998</v>
       </c>
@@ -795,7 +796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>1999</v>
       </c>
@@ -815,7 +816,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>2000</v>
       </c>
@@ -835,7 +836,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>2001</v>
       </c>
@@ -855,7 +856,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>2002</v>
       </c>
@@ -875,7 +876,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>2003</v>
       </c>
@@ -895,7 +896,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>2004</v>
       </c>
@@ -915,7 +916,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>2005</v>
       </c>
@@ -935,7 +936,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>2006</v>
       </c>
@@ -955,7 +956,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>2007</v>
       </c>
@@ -975,7 +976,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>2008</v>
       </c>
@@ -995,7 +996,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>2009</v>
       </c>
@@ -1015,7 +1016,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>2010</v>
       </c>
@@ -1035,7 +1036,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>2011</v>
       </c>
@@ -1055,7 +1056,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>2012</v>
       </c>
@@ -1068,18 +1069,18 @@
       <c r="D30" s="7">
         <v>27731</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="7">
         <v>308</v>
       </c>
       <c r="F30" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>2013</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="7">
         <v>7960</v>
       </c>
       <c r="C31" s="7">
@@ -1088,18 +1089,18 @@
       <c r="D31" s="7">
         <v>13372</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="7">
         <v>785</v>
       </c>
       <c r="F31" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>2014</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="7">
         <v>7066</v>
       </c>
       <c r="C32" s="7">
@@ -1108,14 +1109,18 @@
       <c r="D32" s="7">
         <v>14805</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="7">
         <v>219</v>
       </c>
       <c r="F32" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
+      <c r="H32" s="4"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>2015</v>
       </c>
@@ -1128,14 +1133,18 @@
       <c r="D33" s="7">
         <v>14715</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="7">
         <v>178</v>
       </c>
       <c r="F33" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="5"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>2016</v>
       </c>
@@ -1148,14 +1157,18 @@
       <c r="D34" s="7">
         <v>26710</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="7">
         <v>1266</v>
       </c>
       <c r="F34" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="6"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>2017</v>
       </c>
@@ -1168,14 +1181,18 @@
       <c r="D35" s="7">
         <v>23633</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="7">
         <v>1957</v>
       </c>
       <c r="F35" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="6"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>2018</v>
       </c>
@@ -1185,38 +1202,73 @@
       <c r="C36" s="7">
         <v>53595</v>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="7">
         <v>28518</v>
       </c>
-      <c r="E36" s="9"/>
+      <c r="E36" s="7">
+        <v>4997</v>
+      </c>
       <c r="F36" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="7"/>
+      <c r="K36" s="9"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>2019</v>
       </c>
       <c r="B37" s="7">
         <v>10777</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="7">
         <v>24247</v>
       </c>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
+      <c r="D37" s="7">
+        <v>20258</v>
+      </c>
+      <c r="E37" s="7"/>
       <c r="F37" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="9"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>2020</v>
       </c>
       <c r="B38" s="7">
         <v>7320</v>
       </c>
+      <c r="C38" s="7">
+        <v>17255</v>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
       <c r="F38" t="s">
+        <v>6</v>
+      </c>
+      <c r="H38" s="7"/>
+      <c r="I38" s="11"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="9"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>2021</v>
+      </c>
+      <c r="B39" s="7">
+        <v>6908</v>
+      </c>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1238,22 +1290,26 @@
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="704f474e-3c68-4b88-93ac-7c86e7119ccc">
+    <SharedWithUsers xmlns="bb5346c7-4824-465f-8383-fa07b8a72e7d">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="df73a49c-2dda-4b56-885b-d5c4de27d4ea">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="25bf28c8-6ae6-42aa-a4b2-d83c9f61aeaa" xsi:nil="true"/>
+    <TaxCatchAll xmlns="bb5346c7-4824-465f-8383-fa07b8a72e7d" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005D5936B3F7732444AFEF1606BFED34DC" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="66c4f20a986c90d249ff2b0825fd64ab">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="704f474e-3c68-4b88-93ac-7c86e7119ccc" xmlns:ns3="25bf28c8-6ae6-42aa-a4b2-d83c9f61aeaa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8ded61bcf60b2d2c26d55bb0b6829199" ns1:_="" ns2:_="" ns3:_="">
-    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
-    <xsd:import namespace="704f474e-3c68-4b88-93ac-7c86e7119ccc"/>
-    <xsd:import namespace="25bf28c8-6ae6-42aa-a4b2-d83c9f61aeaa"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CAA43B1AC107724F9284AFB7176B8998" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dd4465f058eaadcba5226029873e111f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="df73a49c-2dda-4b56-885b-d5c4de27d4ea" xmlns:ns3="bb5346c7-4824-465f-8383-fa07b8a72e7d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1b495a1fb07ad1264040cde2ce4afd1a" ns2:_="" ns3:_="">
+    <xsd:import namespace="df73a49c-2dda-4b56-885b-d5c4de27d4ea"/>
+    <xsd:import namespace="bb5346c7-4824-465f-8383-fa07b8a72e7d"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -1262,21 +1318,15 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyProperties" minOccurs="0"/>
-                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyUIAction" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -1284,21 +1334,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="_ip_UnifiedCompliancePolicyProperties" ma:index="15" nillable="true" ma:displayName="Unified Compliance Policy Properties" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyProperties">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="_ip_UnifiedCompliancePolicyUIAction" ma:index="16" nillable="true" ma:displayName="Unified Compliance Policy UI Action" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyUIAction">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="704f474e-3c68-4b88-93ac-7c86e7119ccc" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="df73a49c-2dda-4b56-885b-d5c4de27d4ea" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -1311,65 +1347,43 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="17" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="22" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="360a6a1c-50a4-4ec0-87e3-f00760ffe76b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="360a6a1c-50a4-4ec0-87e3-f00760ffe76b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="18" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="19" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="25bf28c8-6ae6-42aa-a4b2-d83c9f61aeaa" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="bb5346c7-4824-465f-8383-fa07b8a72e7d" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="11" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -1388,14 +1402,14 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="12" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{ccd10a6d-abc8-424f-81e4-b9b81fce80c4}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="25bf28c8-6ae6-42aa-a4b2-d83c9f61aeaa">
+    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3740d791-b6c6-4411-b65f-9ef0a2707c35}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="bb5346c7-4824-465f-8383-fa07b8a72e7d">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -1507,13 +1521,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1C51317-77AF-4EC6-BBCD-D186C6F03BB2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1C51317-77AF-4EC6-BBCD-D186C6F03BB2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8A95344-D05B-435A-9092-07831C2B738C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8A95344-D05B-435A-9092-07831C2B738C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb5346c7-4824-465f-8383-fa07b8a72e7d"/>
+    <ds:schemaRef ds:uri="df73a49c-2dda-4b56-885b-d5c4de27d4ea"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C430EF18-5893-47F9-AC85-2942B5E894F2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7677D28B-31B9-49F4-BD24-B4E65665EB9A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="df73a49c-2dda-4b56-885b-d5c4de27d4ea"/>
+    <ds:schemaRef ds:uri="bb5346c7-4824-465f-8383-fa07b8a72e7d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>